<commit_message>
Deployed 6dd76ba with MkDocs version: 1.6.1
</commit_message>
<xml_diff>
--- a/downloads/acces-date-creation.xlsx
+++ b/downloads/acces-date-creation.xlsx
@@ -10,7 +10,7 @@
     <sheet name="Données" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Données'!$A$1:$C$4</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Données'!$A$1:$C$5</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -425,10 +425,10 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C4"/>
+  <dimension ref="A1:C5"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="18" customWidth="1" min="1" max="1"/>
+    <col width="12" customWidth="1" min="1" max="1"/>
     <col width="14" customWidth="1" min="2" max="2"/>
     <col width="17" customWidth="1" min="3" max="3"/>
   </cols>
@@ -453,44 +453,57 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>Avant 1960</t>
+          <t>1867–1977</t>
         </is>
       </c>
       <c r="B2" t="n">
-        <v>6</v>
+        <v>14</v>
       </c>
       <c r="C2" t="n">
-        <v>17</v>
+        <v>34</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>1960–1999</t>
+          <t>1978–1996</t>
         </is>
       </c>
       <c r="B3" t="n">
-        <v>38</v>
+        <v>23</v>
       </c>
       <c r="C3" t="n">
-        <v>46</v>
+        <v>25</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>À partir de 2000</t>
+          <t>1997–2009</t>
         </is>
       </c>
       <c r="B4" t="n">
-        <v>60</v>
+        <v>28</v>
       </c>
       <c r="C4" t="n">
-        <v>25</v>
+        <v>19</v>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>2010–2025</t>
+        </is>
+      </c>
+      <c r="B5" t="n">
+        <v>39</v>
+      </c>
+      <c r="C5" t="n">
+        <v>10</v>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:C4"/>
+  <autoFilter ref="A1:C5"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Deployed a829544 with MkDocs version: 1.6.1
</commit_message>
<xml_diff>
--- a/downloads/acces-date-creation.xlsx
+++ b/downloads/acces-date-creation.xlsx
@@ -457,36 +457,36 @@
         </is>
       </c>
       <c r="B2" t="n">
-        <v>14</v>
+        <v>15</v>
       </c>
       <c r="C2" t="n">
-        <v>34</v>
+        <v>33</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>1978–1996</t>
+          <t>1978–1995</t>
         </is>
       </c>
       <c r="B3" t="n">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="C3" t="n">
-        <v>25</v>
+        <v>27</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>1997–2009</t>
+          <t>1996–2009</t>
         </is>
       </c>
       <c r="B4" t="n">
-        <v>28</v>
+        <v>31</v>
       </c>
       <c r="C4" t="n">
-        <v>19</v>
+        <v>17</v>
       </c>
     </row>
     <row r="5">
@@ -496,10 +496,10 @@
         </is>
       </c>
       <c r="B5" t="n">
-        <v>39</v>
+        <v>40</v>
       </c>
       <c r="C5" t="n">
-        <v>10</v>
+        <v>11</v>
       </c>
     </row>
   </sheetData>

</xml_diff>